<commit_message>
4 asansör kabini var, ilk asansör harici çok çalışmıyor, asansör kabininin kayması düzgün değil
</commit_message>
<xml_diff>
--- a/elevator_simulation/bin/Debug/net8.0-windows/ml_training_data.xlsx
+++ b/elevator_simulation/bin/Debug/net8.0-windows/ml_training_data.xlsx
@@ -98,6 +98,24 @@
   </x:si>
   <x:si>
     <x:t>23:45:00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-01-19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-02-20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Asansör 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Asansör 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Asansör 4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Asansör 3</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -483,7 +501,7 @@
   <x:dimension ref="A1:I1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:9">
+    <x:row r="1" spans="1:12">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -512,7 +530,7 @@
         <x:v>8</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:9">
+    <x:row r="2" spans="1:12">
       <x:c r="A2" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -541,7 +559,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:9">
+    <x:row r="3" spans="1:12">
       <x:c r="A3" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -570,7 +588,7 @@
         <x:v>12</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:9">
+    <x:row r="4" spans="1:12">
       <x:c r="A4" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -599,7 +617,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:9">
+    <x:row r="5" spans="1:12">
       <x:c r="A5" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -628,7 +646,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" spans="1:9">
+    <x:row r="6" spans="1:12">
       <x:c r="A6" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -657,7 +675,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:9">
+    <x:row r="7" spans="1:12">
       <x:c r="A7" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -686,7 +704,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" spans="1:9">
+    <x:row r="8" spans="1:12">
       <x:c r="A8" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -715,7 +733,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" spans="1:9">
+    <x:row r="9" spans="1:12">
       <x:c r="A9" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -744,7 +762,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" spans="1:9">
+    <x:row r="10" spans="1:12">
       <x:c r="A10" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -773,7 +791,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" spans="1:9">
+    <x:row r="11" spans="1:12">
       <x:c r="A11" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -802,7 +820,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" spans="1:9">
+    <x:row r="12" spans="1:12">
       <x:c r="A12" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -831,7 +849,7 @@
         <x:v>12</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" spans="1:9">
+    <x:row r="13" spans="1:12">
       <x:c r="A13" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -860,7 +878,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" spans="1:9">
+    <x:row r="14" spans="1:12">
       <x:c r="A14" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -889,7 +907,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" spans="1:9">
+    <x:row r="15" spans="1:12">
       <x:c r="A15" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -918,7 +936,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" spans="1:9">
+    <x:row r="16" spans="1:12">
       <x:c r="A16" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -947,7 +965,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" spans="1:9">
+    <x:row r="17" spans="1:12">
       <x:c r="A17" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -976,7 +994,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" spans="1:9">
+    <x:row r="18" spans="1:12">
       <x:c r="A18" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1005,7 +1023,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" spans="1:9">
+    <x:row r="19" spans="1:12">
       <x:c r="A19" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1034,7 +1052,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" spans="1:9">
+    <x:row r="20" spans="1:12">
       <x:c r="A20" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1063,7 +1081,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" spans="1:9">
+    <x:row r="21" spans="1:12">
       <x:c r="A21" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1092,7 +1110,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" spans="1:9">
+    <x:row r="22" spans="1:12">
       <x:c r="A22" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1121,7 +1139,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" spans="1:9">
+    <x:row r="23" spans="1:12">
       <x:c r="A23" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1150,7 +1168,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" spans="1:9">
+    <x:row r="24" spans="1:12">
       <x:c r="A24" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1179,7 +1197,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" spans="1:9">
+    <x:row r="25" spans="1:12">
       <x:c r="A25" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1208,7 +1226,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" spans="1:9">
+    <x:row r="26" spans="1:12">
       <x:c r="A26" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1237,7 +1255,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" spans="1:9">
+    <x:row r="27" spans="1:12">
       <x:c r="A27" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1266,7 +1284,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" spans="1:9">
+    <x:row r="28" spans="1:12">
       <x:c r="A28" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1295,7 +1313,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" spans="1:9">
+    <x:row r="29" spans="1:12">
       <x:c r="A29" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1324,7 +1342,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" spans="1:9">
+    <x:row r="30" spans="1:12">
       <x:c r="A30" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1353,7 +1371,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" spans="1:9">
+    <x:row r="31" spans="1:12">
       <x:c r="A31" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1382,7 +1400,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" spans="1:9">
+    <x:row r="32" spans="1:12">
       <x:c r="A32" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1411,7 +1429,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" spans="1:9">
+    <x:row r="33" spans="1:12">
       <x:c r="A33" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1440,7 +1458,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" spans="1:9">
+    <x:row r="34" spans="1:12">
       <x:c r="A34" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1469,7 +1487,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" spans="1:9">
+    <x:row r="35" spans="1:12">
       <x:c r="A35" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1498,7 +1516,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" spans="1:9">
+    <x:row r="36" spans="1:12">
       <x:c r="A36" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1527,7 +1545,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" spans="1:9">
+    <x:row r="37" spans="1:12">
       <x:c r="A37" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1556,7 +1574,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" spans="1:9">
+    <x:row r="38" spans="1:12">
       <x:c r="A38" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1585,7 +1603,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" spans="1:9">
+    <x:row r="39" spans="1:12">
       <x:c r="A39" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1614,7 +1632,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" spans="1:9">
+    <x:row r="40" spans="1:12">
       <x:c r="A40" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1643,7 +1661,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" spans="1:9">
+    <x:row r="41" spans="1:12">
       <x:c r="A41" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1672,7 +1690,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" spans="1:9">
+    <x:row r="42" spans="1:12">
       <x:c r="A42" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1701,7 +1719,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" spans="1:9">
+    <x:row r="43" spans="1:12">
       <x:c r="A43" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1730,7 +1748,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" spans="1:9">
+    <x:row r="44" spans="1:12">
       <x:c r="A44" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1759,7 +1777,7 @@
         <x:v>21</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" spans="1:9">
+    <x:row r="45" spans="1:12">
       <x:c r="A45" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1788,7 +1806,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" spans="1:9">
+    <x:row r="46" spans="1:12">
       <x:c r="A46" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1817,7 +1835,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" spans="1:9">
+    <x:row r="47" spans="1:12">
       <x:c r="A47" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1846,7 +1864,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="48" spans="1:9">
+    <x:row r="48" spans="1:12">
       <x:c r="A48" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1875,7 +1893,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" spans="1:9">
+    <x:row r="49" spans="1:12">
       <x:c r="A49" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1904,7 +1922,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" spans="1:9">
+    <x:row r="50" spans="1:12">
       <x:c r="A50" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1933,7 +1951,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" spans="1:9">
+    <x:row r="51" spans="1:12">
       <x:c r="A51" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1962,7 +1980,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" spans="1:9">
+    <x:row r="52" spans="1:12">
       <x:c r="A52" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -1991,7 +2009,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="53" spans="1:9">
+    <x:row r="53" spans="1:12">
       <x:c r="A53" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2020,7 +2038,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" spans="1:9">
+    <x:row r="54" spans="1:12">
       <x:c r="A54" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2049,7 +2067,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="55" spans="1:9">
+    <x:row r="55" spans="1:12">
       <x:c r="A55" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2078,7 +2096,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="56" spans="1:9">
+    <x:row r="56" spans="1:12">
       <x:c r="A56" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2107,7 +2125,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" spans="1:9">
+    <x:row r="57" spans="1:12">
       <x:c r="A57" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2136,7 +2154,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="58" spans="1:9">
+    <x:row r="58" spans="1:12">
       <x:c r="A58" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2165,7 +2183,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="59" spans="1:9">
+    <x:row r="59" spans="1:12">
       <x:c r="A59" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2194,7 +2212,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" spans="1:9">
+    <x:row r="60" spans="1:12">
       <x:c r="A60" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2223,7 +2241,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" spans="1:9">
+    <x:row r="61" spans="1:12">
       <x:c r="A61" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2252,7 +2270,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="62" spans="1:9">
+    <x:row r="62" spans="1:12">
       <x:c r="A62" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2281,7 +2299,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="63" spans="1:9">
+    <x:row r="63" spans="1:12">
       <x:c r="A63" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2310,7 +2328,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="64" spans="1:9">
+    <x:row r="64" spans="1:12">
       <x:c r="A64" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2339,7 +2357,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="65" spans="1:9">
+    <x:row r="65" spans="1:12">
       <x:c r="A65" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2368,7 +2386,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" spans="1:9">
+    <x:row r="66" spans="1:12">
       <x:c r="A66" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2397,7 +2415,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" spans="1:9">
+    <x:row r="67" spans="1:12">
       <x:c r="A67" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2426,7 +2444,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" spans="1:9">
+    <x:row r="68" spans="1:12">
       <x:c r="A68" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2455,7 +2473,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" spans="1:9">
+    <x:row r="69" spans="1:12">
       <x:c r="A69" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2484,7 +2502,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" spans="1:9">
+    <x:row r="70" spans="1:12">
       <x:c r="A70" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2513,7 +2531,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" spans="1:9">
+    <x:row r="71" spans="1:12">
       <x:c r="A71" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2542,7 +2560,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" spans="1:9">
+    <x:row r="72" spans="1:12">
       <x:c r="A72" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2571,7 +2589,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" spans="1:9">
+    <x:row r="73" spans="1:12">
       <x:c r="A73" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2600,7 +2618,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" spans="1:9">
+    <x:row r="74" spans="1:12">
       <x:c r="A74" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2629,7 +2647,7 @@
         <x:v>21</x:v>
       </x:c>
     </x:row>
-    <x:row r="75" spans="1:9">
+    <x:row r="75" spans="1:12">
       <x:c r="A75" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2658,7 +2676,7 @@
         <x:v>21</x:v>
       </x:c>
     </x:row>
-    <x:row r="76" spans="1:9">
+    <x:row r="76" spans="1:12">
       <x:c r="A76" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2687,7 +2705,7 @@
         <x:v>21</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" spans="1:9">
+    <x:row r="77" spans="1:12">
       <x:c r="A77" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2716,7 +2734,7 @@
         <x:v>21</x:v>
       </x:c>
     </x:row>
-    <x:row r="78" spans="1:9">
+    <x:row r="78" spans="1:12">
       <x:c r="A78" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2745,7 +2763,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" spans="1:9">
+    <x:row r="79" spans="1:12">
       <x:c r="A79" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2774,7 +2792,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="80" spans="1:9">
+    <x:row r="80" spans="1:12">
       <x:c r="A80" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2803,7 +2821,7 @@
         <x:v>16</x:v>
       </x:c>
     </x:row>
-    <x:row r="81" spans="1:9">
+    <x:row r="81" spans="1:12">
       <x:c r="A81" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2832,7 +2850,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="82" spans="1:9">
+    <x:row r="82" spans="1:12">
       <x:c r="A82" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2861,7 +2879,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" spans="1:9">
+    <x:row r="83" spans="1:12">
       <x:c r="A83" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2890,7 +2908,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="84" spans="1:9">
+    <x:row r="84" spans="1:12">
       <x:c r="A84" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2919,7 +2937,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="85" spans="1:9">
+    <x:row r="85" spans="1:12">
       <x:c r="A85" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2948,7 +2966,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="86" spans="1:9">
+    <x:row r="86" spans="1:12">
       <x:c r="A86" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -2977,7 +2995,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="87" spans="1:9">
+    <x:row r="87" spans="1:12">
       <x:c r="A87" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -3006,7 +3024,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="88" spans="1:9">
+    <x:row r="88" spans="1:12">
       <x:c r="A88" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -3035,7 +3053,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="89" spans="1:9">
+    <x:row r="89" spans="1:12">
       <x:c r="A89" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -3064,7 +3082,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="90" spans="1:9">
+    <x:row r="90" spans="1:12">
       <x:c r="A90" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -3093,7 +3111,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="91" spans="1:9">
+    <x:row r="91" spans="1:12">
       <x:c r="A91" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
@@ -3122,7 +3140,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" spans="1:9">
+    <x:row r="92" spans="1:12">
       <x:c r="A92" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3151,7 +3169,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" spans="1:9">
+    <x:row r="93" spans="1:12">
       <x:c r="A93" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3180,7 +3198,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" spans="1:9">
+    <x:row r="94" spans="1:12">
       <x:c r="A94" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3209,7 +3227,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" spans="1:9">
+    <x:row r="95" spans="1:12">
       <x:c r="A95" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3238,7 +3256,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="96" spans="1:9">
+    <x:row r="96" spans="1:12">
       <x:c r="A96" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3267,7 +3285,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="97" spans="1:9">
+    <x:row r="97" spans="1:12">
       <x:c r="A97" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3296,7 +3314,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="98" spans="1:9">
+    <x:row r="98" spans="1:12">
       <x:c r="A98" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3325,7 +3343,7 @@
         <x:v>13</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" spans="1:9">
+    <x:row r="99" spans="1:12">
       <x:c r="A99" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3354,7 +3372,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" spans="1:9">
+    <x:row r="100" spans="1:12">
       <x:c r="A100" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3383,7 +3401,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" spans="1:9">
+    <x:row r="101" spans="1:12">
       <x:c r="A101" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3412,7 +3430,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" spans="1:9">
+    <x:row r="102" spans="1:12">
       <x:c r="A102" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3441,7 +3459,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" spans="1:9">
+    <x:row r="103" spans="1:12">
       <x:c r="A103" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3470,7 +3488,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" spans="1:9">
+    <x:row r="104" spans="1:12">
       <x:c r="A104" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3499,7 +3517,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" spans="1:9">
+    <x:row r="105" spans="1:12">
       <x:c r="A105" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3528,7 +3546,7 @@
         <x:v>12</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" spans="1:9">
+    <x:row r="106" spans="1:12">
       <x:c r="A106" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3557,7 +3575,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" spans="1:9">
+    <x:row r="107" spans="1:12">
       <x:c r="A107" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3586,7 +3604,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="108" spans="1:9">
+    <x:row r="108" spans="1:12">
       <x:c r="A108" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3615,7 +3633,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" spans="1:9">
+    <x:row r="109" spans="1:12">
       <x:c r="A109" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3644,7 +3662,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="110" spans="1:9">
+    <x:row r="110" spans="1:12">
       <x:c r="A110" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3673,7 +3691,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="111" spans="1:9">
+    <x:row r="111" spans="1:12">
       <x:c r="A111" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3702,7 +3720,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="112" spans="1:9">
+    <x:row r="112" spans="1:12">
       <x:c r="A112" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3731,7 +3749,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="113" spans="1:9">
+    <x:row r="113" spans="1:12">
       <x:c r="A113" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3760,7 +3778,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="114" spans="1:9">
+    <x:row r="114" spans="1:12">
       <x:c r="A114" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3789,7 +3807,7 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
-    <x:row r="115" spans="1:9">
+    <x:row r="115" spans="1:12">
       <x:c r="A115" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3818,7 +3836,7 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="116" spans="1:9">
+    <x:row r="116" spans="1:12">
       <x:c r="A116" s="2" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -3844,6 +3862,2769 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I116" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" spans="1:12">
+      <x:c r="A117" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B117" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C117" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D117" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E117" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F117" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G117" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H117" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I117" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" spans="1:12">
+      <x:c r="A118" s="2" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B118" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C118" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D118" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E118" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F118" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G118" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H118" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I118" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" spans="1:12">
+      <x:c r="A119" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B119" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C119" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D119" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E119" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F119" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G119" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H119" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I119" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" spans="1:12">
+      <x:c r="A120" s="2" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B120" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C120" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D120" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E120" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F120" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G120" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H120" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I120" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" spans="1:12">
+      <x:c r="A121" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B121" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C121" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D121" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E121" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F121" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G121" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H121" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I121" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" spans="1:12">
+      <x:c r="A122" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B122" s="2" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C122" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D122" s="2">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E122" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F122" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G122" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H122" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I122" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" spans="1:12">
+      <x:c r="A123" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B123" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C123" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D123" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E123" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F123" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G123" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H123" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I123" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" spans="1:12">
+      <x:c r="A124" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B124" s="2" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C124" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D124" s="2">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E124" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F124" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G124" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H124" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I124" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" spans="1:12">
+      <x:c r="A125" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B125" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C125" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D125" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E125" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F125" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G125" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H125" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I125" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" spans="1:12">
+      <x:c r="A126" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B126" s="2" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C126" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D126" s="2">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E126" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F126" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G126" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H126" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I126" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" spans="1:12">
+      <x:c r="A127" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B127" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C127" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D127" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E127" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F127" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G127" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H127" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I127" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" spans="1:12">
+      <x:c r="A128" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B128" s="2" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C128" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D128" s="2">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E128" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F128" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G128" s="2">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H128" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I128" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" spans="1:12">
+      <x:c r="A129" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B129" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C129" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D129" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E129" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F129" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G129" s="0">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H129" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I129" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" spans="1:12">
+      <x:c r="A130" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B130" s="2" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C130" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D130" s="2">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E130" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F130" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G130" s="2">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H130" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I130" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" spans="1:12">
+      <x:c r="A131" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B131" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C131" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D131" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E131" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F131" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G131" s="0">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H131" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I131" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" spans="1:12">
+      <x:c r="A132" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B132" s="2" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C132" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D132" s="2">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E132" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F132" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G132" s="2">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="H132" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I132" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" spans="1:12">
+      <x:c r="A133" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B133" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C133" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D133" s="0">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E133" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F133" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G133" s="0">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H133" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I133" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134" spans="1:12">
+      <x:c r="A134" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B134" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C134" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D134" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E134" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F134" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G134" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H134" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I134" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135" spans="1:12">
+      <x:c r="A135" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B135" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C135" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D135" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E135" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F135" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G135" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H135" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I135" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" spans="1:12">
+      <x:c r="A136" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B136" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C136" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D136" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E136" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F136" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G136" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H136" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I136" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137" spans="1:12">
+      <x:c r="A137" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B137" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C137" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D137" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E137" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F137" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G137" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H137" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I137" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" spans="1:12">
+      <x:c r="A138" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B138" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C138" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D138" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E138" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F138" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G138" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H138" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I138" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" spans="1:12">
+      <x:c r="A139" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B139" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C139" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D139" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E139" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F139" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G139" s="0">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H139" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I139" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" spans="1:12">
+      <x:c r="A140" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B140" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C140" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D140" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E140" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F140" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G140" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H140" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I140" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" spans="1:12">
+      <x:c r="A141" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B141" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C141" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D141" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E141" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F141" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G141" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H141" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I141" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" spans="1:12">
+      <x:c r="A142" s="2" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B142" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C142" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D142" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E142" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F142" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G142" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H142" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I142" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" spans="1:12">
+      <x:c r="A143" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B143" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C143" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D143" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E143" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F143" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G143" s="0">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H143" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I143" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" spans="1:12">
+      <x:c r="A144" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B144" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C144" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D144" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E144" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F144" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G144" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H144" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I144" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" spans="1:12">
+      <x:c r="A145" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B145" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C145" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D145" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E145" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F145" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G145" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H145" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I145" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" spans="1:12">
+      <x:c r="A146" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B146" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C146" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D146" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E146" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F146" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G146" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H146" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I146" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" spans="1:12">
+      <x:c r="A147" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B147" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C147" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D147" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E147" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F147" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G147" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H147" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I147" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" spans="1:12">
+      <x:c r="A148" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B148" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C148" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D148" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E148" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F148" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G148" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H148" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I148" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" spans="1:12">
+      <x:c r="A149" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B149" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C149" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D149" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E149" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F149" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G149" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H149" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I149" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" spans="1:12">
+      <x:c r="A150" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B150" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C150" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D150" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E150" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F150" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G150" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H150" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I150" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" spans="1:12">
+      <x:c r="A151" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B151" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C151" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D151" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E151" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F151" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G151" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H151" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I151" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" spans="1:12">
+      <x:c r="A152" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B152" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C152" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D152" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E152" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F152" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G152" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H152" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I152" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J152" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K152" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L152" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" spans="1:12">
+      <x:c r="A153" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B153" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C153" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D153" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E153" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F153" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G153" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H153" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I153" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J153" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K153" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L153" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" spans="1:12">
+      <x:c r="A154" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B154" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C154" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D154" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E154" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F154" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G154" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H154" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I154" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J154" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K154" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L154" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" spans="1:12">
+      <x:c r="A155" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B155" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C155" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D155" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E155" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F155" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G155" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H155" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I155" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J155" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K155" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L155" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" spans="1:12">
+      <x:c r="A156" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B156" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C156" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D156" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E156" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F156" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G156" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H156" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I156" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J156" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K156" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L156" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" spans="1:12">
+      <x:c r="A157" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B157" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C157" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D157" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E157" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F157" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G157" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H157" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I157" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J157" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K157" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L157" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" spans="1:12">
+      <x:c r="A158" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B158" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C158" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D158" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E158" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F158" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G158" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H158" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I158" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J158" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K158" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L158" s="2" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" spans="1:12">
+      <x:c r="A159" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B159" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C159" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D159" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E159" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F159" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G159" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H159" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I159" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J159" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K159" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L159" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" spans="1:12">
+      <x:c r="A160" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B160" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C160" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D160" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E160" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F160" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G160" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H160" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I160" s="2" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J160" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K160" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L160" s="2" t="s">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" spans="1:12">
+      <x:c r="A161" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B161" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C161" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D161" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E161" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F161" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G161" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H161" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I161" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J161" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K161" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L161" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" spans="1:12">
+      <x:c r="A162" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B162" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C162" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D162" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E162" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F162" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G162" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H162" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I162" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J162" s="2">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K162" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L162" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" spans="1:12">
+      <x:c r="A163" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B163" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C163" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D163" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E163" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F163" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G163" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H163" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I163" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J163" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K163" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L163" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" spans="1:12">
+      <x:c r="A164" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B164" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C164" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D164" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E164" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F164" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G164" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H164" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I164" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J164" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K164" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L164" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" spans="1:12">
+      <x:c r="A165" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B165" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C165" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D165" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E165" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F165" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G165" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H165" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I165" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J165" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K165" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L165" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" spans="1:12">
+      <x:c r="A166" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B166" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C166" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D166" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E166" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F166" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G166" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H166" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I166" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J166" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K166" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L166" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" spans="1:12">
+      <x:c r="A167" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B167" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C167" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D167" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E167" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F167" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G167" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H167" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I167" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J167" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K167" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L167" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" spans="1:12">
+      <x:c r="A168" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B168" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C168" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D168" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E168" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F168" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G168" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H168" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I168" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J168" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K168" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L168" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" spans="1:12">
+      <x:c r="A169" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B169" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C169" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D169" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E169" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F169" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G169" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H169" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I169" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J169" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K169" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L169" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" spans="1:12">
+      <x:c r="A170" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B170" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C170" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D170" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E170" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F170" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G170" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H170" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I170" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J170" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K170" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L170" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" spans="1:12">
+      <x:c r="A171" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B171" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C171" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D171" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E171" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F171" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G171" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H171" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I171" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J171" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K171" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L171" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" spans="1:12">
+      <x:c r="A172" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B172" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C172" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D172" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E172" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F172" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G172" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H172" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I172" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J172" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K172" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L172" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" spans="1:12">
+      <x:c r="A173" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B173" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C173" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D173" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E173" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F173" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G173" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H173" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I173" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J173" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K173" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L173" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" spans="1:12">
+      <x:c r="A174" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B174" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C174" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D174" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E174" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F174" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G174" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H174" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I174" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J174" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K174" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L174" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" spans="1:12">
+      <x:c r="A175" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B175" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C175" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D175" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E175" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F175" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G175" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H175" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I175" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J175" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K175" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L175" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" spans="1:12">
+      <x:c r="A176" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B176" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C176" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D176" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E176" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F176" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G176" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H176" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I176" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J176" s="2">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K176" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L176" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" spans="1:12">
+      <x:c r="A177" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B177" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C177" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D177" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E177" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F177" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G177" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H177" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I177" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J177" s="0">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K177" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L177" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" spans="1:12">
+      <x:c r="A178" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B178" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C178" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D178" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E178" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F178" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G178" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H178" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I178" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J178" s="2">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K178" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L178" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" spans="1:12">
+      <x:c r="A179" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B179" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C179" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D179" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E179" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F179" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G179" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H179" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I179" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J179" s="0">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K179" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L179" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" spans="1:12">
+      <x:c r="A180" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B180" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C180" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D180" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E180" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F180" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G180" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H180" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I180" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J180" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K180" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L180" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" spans="1:12">
+      <x:c r="A181" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B181" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C181" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D181" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E181" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F181" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G181" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H181" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I181" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J181" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K181" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L181" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" spans="1:12">
+      <x:c r="A182" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B182" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C182" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D182" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E182" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F182" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G182" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H182" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I182" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J182" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K182" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L182" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" spans="1:12">
+      <x:c r="A183" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B183" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C183" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D183" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E183" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F183" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G183" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H183" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I183" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J183" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K183" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L183" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" spans="1:12">
+      <x:c r="A184" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B184" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C184" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D184" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E184" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F184" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G184" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H184" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I184" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J184" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K184" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L184" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" spans="1:12">
+      <x:c r="A185" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B185" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C185" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D185" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E185" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F185" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G185" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H185" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I185" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J185" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K185" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L185" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" spans="1:12">
+      <x:c r="A186" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B186" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C186" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D186" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E186" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F186" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G186" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H186" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I186" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J186" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K186" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L186" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" spans="1:12">
+      <x:c r="A187" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B187" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C187" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D187" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E187" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F187" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G187" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H187" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I187" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J187" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K187" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L187" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" spans="1:12">
+      <x:c r="A188" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B188" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C188" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D188" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E188" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F188" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G188" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H188" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I188" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J188" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K188" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L188" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" spans="1:12">
+      <x:c r="A189" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B189" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C189" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D189" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E189" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F189" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G189" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H189" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I189" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J189" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K189" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L189" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" spans="1:12">
+      <x:c r="A190" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B190" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C190" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D190" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E190" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F190" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G190" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H190" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I190" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J190" s="2">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K190" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L190" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" spans="1:12">
+      <x:c r="A191" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B191" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C191" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D191" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E191" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F191" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G191" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H191" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I191" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J191" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K191" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L191" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" spans="1:12">
+      <x:c r="A192" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B192" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C192" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D192" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E192" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F192" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G192" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H192" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I192" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J192" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K192" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L192" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" spans="1:12">
+      <x:c r="A193" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B193" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C193" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D193" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E193" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F193" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G193" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H193" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I193" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J193" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K193" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L193" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" spans="1:12">
+      <x:c r="A194" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B194" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C194" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D194" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E194" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F194" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G194" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H194" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I194" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J194" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K194" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L194" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" spans="1:12">
+      <x:c r="A195" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B195" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C195" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D195" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E195" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F195" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G195" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H195" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I195" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J195" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K195" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L195" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" spans="1:12">
+      <x:c r="A196" s="2" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B196" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C196" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D196" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E196" s="2">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F196" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G196" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H196" s="2">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I196" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J196" s="2">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K196" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L196" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" spans="1:12">
+      <x:c r="A197" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B197" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C197" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D197" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E197" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F197" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G197" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H197" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I197" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J197" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K197" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L197" s="0" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
3.ve 4. asansör için de kat çizgileri eklendi fakat katlar arkada kaymıyoe iç tuş takımı da düzensiz
</commit_message>
<xml_diff>
--- a/elevator_simulation/bin/Debug/net8.0-windows/ml_training_data.xlsx
+++ b/elevator_simulation/bin/Debug/net8.0-windows/ml_training_data.xlsx
@@ -116,6 +116,9 @@
   </x:si>
   <x:si>
     <x:t>Asansör 3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-02-28</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -6628,6 +6631,880 @@
         <x:v>14</x:v>
       </x:c>
     </x:row>
+    <x:row r="198" spans="1:12">
+      <x:c r="A198" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B198" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C198" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D198" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E198" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F198" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G198" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H198" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I198" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J198" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K198" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L198" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" spans="1:12">
+      <x:c r="A199" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B199" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C199" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D199" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E199" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F199" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G199" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H199" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I199" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J199" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K199" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L199" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="200" spans="1:12">
+      <x:c r="A200" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B200" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C200" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D200" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E200" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F200" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G200" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H200" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I200" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J200" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K200" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L200" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" spans="1:12">
+      <x:c r="A201" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B201" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C201" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D201" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E201" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F201" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G201" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H201" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I201" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J201" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K201" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L201" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" spans="1:12">
+      <x:c r="A202" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B202" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C202" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D202" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E202" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F202" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G202" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H202" s="2">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I202" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J202" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K202" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L202" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" spans="1:12">
+      <x:c r="A203" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B203" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C203" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D203" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E203" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F203" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G203" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H203" s="0">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I203" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J203" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K203" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L203" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" spans="1:12">
+      <x:c r="A204" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B204" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C204" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D204" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E204" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F204" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G204" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H204" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I204" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J204" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K204" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L204" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" spans="1:12">
+      <x:c r="A205" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B205" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C205" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D205" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E205" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F205" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G205" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H205" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I205" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J205" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K205" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L205" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" spans="1:12">
+      <x:c r="A206" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B206" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C206" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D206" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E206" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F206" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G206" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H206" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I206" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J206" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K206" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L206" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" spans="1:12">
+      <x:c r="A207" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B207" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C207" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D207" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E207" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F207" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G207" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H207" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I207" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J207" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K207" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L207" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" spans="1:12">
+      <x:c r="A208" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B208" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C208" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D208" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E208" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F208" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G208" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H208" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I208" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J208" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K208" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L208" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" spans="1:12">
+      <x:c r="A209" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B209" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C209" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D209" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E209" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F209" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G209" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H209" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I209" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J209" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K209" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L209" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" spans="1:12">
+      <x:c r="A210" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B210" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C210" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D210" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E210" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F210" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G210" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H210" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I210" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J210" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K210" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L210" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" spans="1:12">
+      <x:c r="A211" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B211" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C211" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D211" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E211" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F211" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G211" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H211" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I211" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J211" s="0">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K211" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L211" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" spans="1:12">
+      <x:c r="A212" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B212" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C212" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D212" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E212" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F212" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G212" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H212" s="2">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I212" s="2" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J212" s="2">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K212" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L212" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="213" spans="1:12">
+      <x:c r="A213" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B213" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C213" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D213" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E213" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F213" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G213" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H213" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I213" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J213" s="0">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="K213" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L213" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" spans="1:12">
+      <x:c r="A214" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B214" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C214" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D214" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E214" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F214" s="2">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G214" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H214" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I214" s="2" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J214" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K214" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L214" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" spans="1:12">
+      <x:c r="A215" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B215" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C215" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D215" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E215" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F215" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G215" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H215" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I215" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="J215" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K215" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L215" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" spans="1:12">
+      <x:c r="A216" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B216" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C216" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D216" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E216" s="2">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F216" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G216" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H216" s="2">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I216" s="2" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J216" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K216" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L216" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" spans="1:12">
+      <x:c r="A217" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B217" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C217" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D217" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E217" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F217" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G217" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H217" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I217" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J217" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K217" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L217" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" spans="1:12">
+      <x:c r="A218" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B218" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C218" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D218" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E218" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F218" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G218" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H218" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I218" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J218" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K218" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L218" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" spans="1:12">
+      <x:c r="A219" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B219" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C219" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D219" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E219" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F219" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G219" s="0">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H219" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I219" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J219" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K219" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L219" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" spans="1:12">
+      <x:c r="A220" s="2" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B220" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C220" s="2">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D220" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E220" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F220" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G220" s="2">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="H220" s="2">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I220" s="2" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="J220" s="2">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K220" s="2">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L220" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>